<commit_message>
fix: keep only the tables and their notes in the Excel workbook
The workbook no longer starts with a sheet describing the file, and prose paragraphs from the page (such as the introduction of the word list) are left out. Sheets now start directly with their first table; notes and sub-headings between tables remain.

Assisted-by: Claude:claude-fable-5
</commit_message>
<xml_diff>
--- a/static/downloads/hebreeuws-braille.xlsx
+++ b/static/downloads/hebreeuws-braille.xlsx
@@ -4,14 +4,13 @@
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Over dit bestand" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Consonanten" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Vocalen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Overige tekens" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Woorden" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Consonanten" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Vocalen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Overige tekens" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Woorden" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -55,11 +54,11 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" readingOrder="2"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment readingOrder="2"/>
     </xf>
@@ -211,8 +210,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Woorden" displayName="Woorden" ref="A3:C28" headerRowCount="1">
-  <autoFilter ref="A3:C28"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="Woorden" displayName="Woorden" ref="A1:C26" headerRowCount="1">
+  <autoFilter ref="A1:C26"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Woord"/>
     <tableColumn id="2" name="Unicode Braille"/>
@@ -511,44 +510,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Hebreeuws</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Op deze pagina is meer te vinden over het Hebreeuws, met name over Hebreeuws braille.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Bron: https://didymus.info/languages/hebrew/</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -560,824 +521,824 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Karakter</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Unicode Braille</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ASCII Braille</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Braillepunten</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>א</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Alef</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>⠁</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>בּ</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Beet met dageesj</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>⠃</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ב</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Beet zonder dageesj</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>⠧</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>v</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>1236</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>גּ</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Gimel met Dageesj</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>⠐⠛</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>"g</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>5-1245</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ג</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Gimel zonder dageesj</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>⠛</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>g</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>1245</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>דּ</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Dalet met dageesj</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>⠐⠙</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>"d</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>5-145</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ד</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Dalet zonder dageesj</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>⠙</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>145</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ה</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Hee</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>⠓</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>125</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ו</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Wav</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>⠺</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>w</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>2456</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ז</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Zajin</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>⠵</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>z</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>1356</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>ח</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Chet</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>⠭</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>1346</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>ט</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Tet</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>⠞</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>t</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>2345</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>י</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Jod</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>⠚</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>j</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>245</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>כּ / ּךּ</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B15" s="1" t="inlineStr">
         <is>
           <t>Kaf met dageesj</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
+      <c r="C15" s="1" t="inlineStr">
         <is>
           <t>⠅</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
+      <c r="D15" s="1" t="inlineStr">
         <is>
           <t>k</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="E15" s="1" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>כ / ך</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B16" s="1" t="inlineStr">
         <is>
           <t>Kaf zonder dageesj</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C16" s="1" t="inlineStr">
         <is>
           <t>⠡</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D16" s="1" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="E16" s="1" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>ל</t>
         </is>
       </c>
-      <c r="B17" s="2" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Lamed</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>⠇</t>
         </is>
       </c>
-      <c r="D17" s="2" t="inlineStr">
+      <c r="D17" s="1" t="inlineStr">
         <is>
           <t>l</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="E17" s="1" t="inlineStr">
         <is>
           <t>123</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>מ / ם</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Mem</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>⠍</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>134</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>נ / ן</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Noen</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>⠝</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>n</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>1345</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>ס</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Samech</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>⠎</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>s</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>234</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>ע</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Ajin</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>⠫</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>1246</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>פּ / ףּ</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Pee met dageesj</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>⠏</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>1234</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>פ / ף</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B23" s="1" t="inlineStr">
         <is>
           <t>Pee zonder dageesj</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C23" s="1" t="inlineStr">
         <is>
           <t>⠋</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D23" s="1" t="inlineStr">
         <is>
           <t>f</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E23" s="1" t="inlineStr">
         <is>
           <t>124</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>צ / ץ</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B24" s="1" t="inlineStr">
         <is>
           <t>Tsadee</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C24" s="1" t="inlineStr">
         <is>
           <t>⠮</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>!</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>2346</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>ק</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
+      <c r="B25" s="1" t="inlineStr">
         <is>
           <t>Kof</t>
         </is>
       </c>
-      <c r="C25" s="2" t="inlineStr">
+      <c r="C25" s="1" t="inlineStr">
         <is>
           <t>⠟</t>
         </is>
       </c>
-      <c r="D25" s="2" t="inlineStr">
+      <c r="D25" s="1" t="inlineStr">
         <is>
           <t>q</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="E25" s="1" t="inlineStr">
         <is>
           <t>12345</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>ר</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>Reesj</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>⠗</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="1" t="inlineStr">
         <is>
           <t>r</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="E26" s="1" t="inlineStr">
         <is>
           <t>1235</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>שׂ</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Sien</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>⠱</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
         <is>
           <t>:</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E27" s="1" t="inlineStr">
         <is>
           <t>156</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>שׁ</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B28" s="1" t="inlineStr">
         <is>
           <t>Sjien</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C28" s="1" t="inlineStr">
         <is>
           <t>⠩</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D28" s="1" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E28" s="1" t="inlineStr">
         <is>
           <t>146</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>תּ</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B29" s="1" t="inlineStr">
         <is>
           <t>Tav met dageesj</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C29" s="1" t="inlineStr">
         <is>
           <t>⠳</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D29" s="1" t="inlineStr">
         <is>
           <t>\</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E29" s="1" t="inlineStr">
         <is>
           <t>1256</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+      <c r="A30" s="2" t="inlineStr">
         <is>
           <t>ת</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B30" s="1" t="inlineStr">
         <is>
           <t>Tav zonder dageesj</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C30" s="1" t="inlineStr">
         <is>
           <t>⠹</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D30" s="1" t="inlineStr">
         <is>
           <t>?</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E30" s="1" t="inlineStr">
         <is>
           <t>1456</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>De Beet, Kaf, Pee en Tav krijgen in braille een apart teken wanneer zij een Dageesj bevatten. Bij andere consonanten (inclusief de Gimel en Dalet) wordt de Dageesj (braillepunt 5, ⠐) vóór de consonant geplaatst.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
+      <c r="A34" s="1" t="inlineStr">
         <is>
           <t>De sluitletters in het Hebreeuwse alfabet worden volgens de IHBC-standaard niet onderscheiden van de normale letters.</t>
         </is>
@@ -1391,7 +1352,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1409,370 +1370,370 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Karakter</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Unicode Braille</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ASCII Braille</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Braillepunten</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ְ</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Sjwa</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>⠄</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>'</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>ִ</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Chirek</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>⠊</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>i</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>ֵ</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Tseree</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>⠌</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>ֶ</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Segol</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>⠑</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>e</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>ֱ</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Chateef segol</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>⠢</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>ַ</t>
         </is>
       </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" s="1" t="inlineStr">
         <is>
           <t>Patach</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>⠉</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>ֲ</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" s="1" t="inlineStr">
         <is>
           <t>Chateef patach</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>⠒</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>ָ</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B9" s="1" t="inlineStr">
         <is>
           <t>Kamets</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>⠣</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
+      <c r="D9" s="1" t="inlineStr">
         <is>
           <t>&lt;</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="E9" s="1" t="inlineStr">
         <is>
           <t>126</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>ֳ</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Chateef kamets</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>⠜</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>&gt;</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>345</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>ֹ</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Cholem</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>⠕</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>o</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>135</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>ֻ</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Kiboets</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>⠥</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>u</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>136</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Leesmoeders</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+      <c r="A16" s="1" t="inlineStr">
         <is>
           <t>Wanneer de letters Wav en Jod fungeren als leesmoeders in plaats van als medeklinkers, worden ze tot één enkele braille-cel samengetrokken.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+      <c r="A18" s="1" t="inlineStr">
         <is>
           <t>Karakter</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="B18" s="1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
+      <c r="C18" s="1" t="inlineStr">
         <is>
           <t>Unicode Braille</t>
         </is>
       </c>
-      <c r="D18" s="2" t="inlineStr">
+      <c r="D18" s="1" t="inlineStr">
         <is>
           <t>ASCII Braille</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="E18" s="1" t="inlineStr">
         <is>
           <t>Braillepunten</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="F18" s="1" t="inlineStr">
         <is>
           <t>Opmerking</t>
         </is>
@@ -1784,27 +1745,27 @@
           <t>ִי</t>
         </is>
       </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="B19" s="1" t="inlineStr">
         <is>
           <t>Chierek-jod</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
+      <c r="C19" s="1" t="inlineStr">
         <is>
           <t>⠔</t>
         </is>
       </c>
-      <c r="D19" s="2" t="inlineStr">
+      <c r="D19" s="1" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="E19" s="1" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="F19" s="1" t="inlineStr">
         <is>
           <t>Verlaagde Chirek</t>
         </is>
@@ -1816,27 +1777,27 @@
           <t>ֵי</t>
         </is>
       </c>
-      <c r="B20" s="2" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Tseree-jod</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>⠼</t>
         </is>
       </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E20" s="1" t="inlineStr">
         <is>
           <t>3456</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="F20" s="1" t="inlineStr">
         <is>
           <t>Combinatie Tseree en verlaagde jod</t>
         </is>
@@ -1848,27 +1809,27 @@
           <t>וֹ</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
+      <c r="B21" s="1" t="inlineStr">
         <is>
           <t>Cholem-wav</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
+      <c r="C21" s="1" t="inlineStr">
         <is>
           <t>⠪</t>
         </is>
       </c>
-      <c r="D21" s="2" t="inlineStr">
+      <c r="D21" s="1" t="inlineStr">
         <is>
           <t>[</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E21" s="1" t="inlineStr">
         <is>
           <t>246</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="F21" s="1" t="inlineStr">
         <is>
           <t>Gespiegelde Cholem</t>
         </is>
@@ -1880,34 +1841,34 @@
           <t>וּ</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B22" s="1" t="inlineStr">
         <is>
           <t>Sjoeroek</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C22" s="1" t="inlineStr">
         <is>
           <t>⠬</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D22" s="1" t="inlineStr">
         <is>
           <t>+</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="E22" s="1" t="inlineStr">
         <is>
           <t>346</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="F22" s="1" t="inlineStr">
         <is>
           <t>Gespiegelde Kiboets</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+      <c r="A24" s="1" t="inlineStr">
         <is>
           <t>De letters Alef en Hee worden niet samengetrokken als ze als leesmoeders worden gebruikt.</t>
         </is>
@@ -1922,7 +1883,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1939,257 +1900,257 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Karakter</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Unicode Braille</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ASCII Braille</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Braillepunten</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>ּ</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="1" t="inlineStr">
         <is>
           <t>Dageesj</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>⠐</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>"</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>הּ</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>Hee met mapiek</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>⠓⠘</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>h^</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>125-45</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>־</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" s="1" t="inlineStr">
         <is>
           <t>Makeef</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>⠤</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>36</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>׀</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" s="1" t="inlineStr">
         <is>
           <t>Paassek</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>⠸</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>_</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>456</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Scheidende accenten</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="1" t="inlineStr">
         <is>
           <t>De onderstaande drie scheidende accenten worden in braille aan het einde van het woord geplaatst waarin ze voorkomen.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="1" t="inlineStr">
         <is>
           <t>Karakter</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Naam</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Unicode Braille</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="D11" s="1" t="inlineStr">
         <is>
           <t>ASCII Braille</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="E11" s="1" t="inlineStr">
         <is>
           <t>Braillepunten</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>֔</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Zakeef katon</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
+      <c r="C12" s="1" t="inlineStr">
         <is>
           <t>⠂</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
+      <c r="D12" s="1" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="E12" s="1" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>֑</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B13" s="1" t="inlineStr">
         <is>
           <t>Atnach</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
+      <c r="C13" s="1" t="inlineStr">
         <is>
           <t>⠆</t>
         </is>
       </c>
-      <c r="D13" s="2" t="inlineStr">
+      <c r="D13" s="1" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="E13" s="1" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="2" t="inlineStr">
         <is>
           <t>׃</t>
         </is>
       </c>
-      <c r="B14" s="2" t="inlineStr">
+      <c r="B14" s="1" t="inlineStr">
         <is>
           <t>Sof pasoek</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
+      <c r="C14" s="1" t="inlineStr">
         <is>
           <t>⠲</t>
         </is>
       </c>
-      <c r="D14" s="2" t="inlineStr">
+      <c r="D14" s="1" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="E14" s="1" t="inlineStr">
         <is>
           <t>256</t>
         </is>
@@ -2204,13 +2165,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2219,449 +2180,442 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Als voorbeeld volgen hieronder een aantal Hebreeuwse woorden met hun representatie in braille. De woorden zijn zo gekozen dat ze zo veel mogelijk braillecombinaties laten zien.</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Woord</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unicode Braille</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>ASCII Braille</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>אָב</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>⠁⠣⠧</t>
+        </is>
+      </c>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>a&lt;v</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Woord</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Unicode Braille</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>ASCII Braille</t>
+          <t>אֱמֶת</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t>⠁⠢⠍⠑⠹</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>a5me?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>אָב</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>⠁⠣⠧</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>a&lt;v</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>בַּת</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>⠃⠉⠹</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>bc?</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>אֱמֶת</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>⠁⠢⠍⠑⠹</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>a5me?</t>
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>גָּדוֹל</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>⠐⠛⠣⠙⠪⠇</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>"g&lt;d[l</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>בַּת</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>⠃⠉⠹</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>bc?</t>
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>דֶּרֶךְ</t>
+        </is>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>⠐⠙⠑⠗⠑⠅⠄</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>"derek'</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>גָּדוֹל</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>⠐⠛⠣⠙⠪⠇</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>"g&lt;d[l</t>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>הֵיכָל</t>
+        </is>
+      </c>
+      <c r="B7" s="1" t="inlineStr">
+        <is>
+          <t>⠓⠼⠡⠣⠇</t>
+        </is>
+      </c>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>h#/&lt;l</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>דֶּרֶךְ</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>⠐⠙⠑⠗⠑⠅⠄</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>"derek'</t>
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>וְ</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>⠺⠄</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>w'</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>הֵיכָל</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>⠓⠼⠡⠣⠇</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>h#/&lt;l</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>זֶרַע</t>
+        </is>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>⠵⠑⠗⠉⠫</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>zerc$</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>וְ</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>⠺⠄</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>w'</t>
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>חֲכָם</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>⠭⠒⠡⠣⠍</t>
+        </is>
+      </c>
+      <c r="C10" s="1" t="inlineStr">
+        <is>
+          <t>x3*&lt;m</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>זֶרַע</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>⠵⠑⠗⠉⠫</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>zerc$</t>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>חֳלִי</t>
+        </is>
+      </c>
+      <c r="B11" s="1" t="inlineStr">
+        <is>
+          <t>⠭⠜⠇⠔</t>
+        </is>
+      </c>
+      <c r="C11" s="1" t="inlineStr">
+        <is>
+          <t>x&gt;l9</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>חֲכָם</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>⠭⠒⠡⠣⠍</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>x3*&lt;m</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>חֵמָה</t>
+        </is>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>⠭⠌⠍⠣⠓</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>x/m&lt;h</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>חֳלִי</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>⠭⠜⠇⠔</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>x&gt;l9</t>
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>טוֹב</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>⠞⠪⠧</t>
+        </is>
+      </c>
+      <c r="C13" s="1" t="inlineStr">
+        <is>
+          <t>t[v</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>חֵמָה</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>⠭⠌⠍⠣⠓</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>x/m&lt;h</t>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>יָמִין</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>⠚⠣⠍⠔⠝</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>j&lt;m9n</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
-        <is>
-          <t>טוֹב</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>⠞⠪⠧</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>t[v</t>
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>כֹּהֵן</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>⠅⠕⠓⠌⠝</t>
+        </is>
+      </c>
+      <c r="C15" s="1" t="inlineStr">
+        <is>
+          <t>koh/n</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>יָמִין</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>⠚⠣⠍⠔⠝</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>j&lt;m9n</t>
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>כָּבוֹד</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>⠅⠣⠧⠪⠙</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>k&lt;v[d</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>כֹּהֵן</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>⠅⠕⠓⠌⠝</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>koh/n</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>לֶחֶם</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>⠇⠑⠭⠑⠍</t>
+        </is>
+      </c>
+      <c r="C17" s="1" t="inlineStr">
+        <is>
+          <t>lexem</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>כָּבוֹד</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>⠅⠣⠧⠪⠙</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>k&lt;v[d</t>
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>מִזְבֵּחַ</t>
+        </is>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>⠍⠊⠵⠄⠃⠌⠭⠉</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>miz'b/xc</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>לֶחֶם</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>⠇⠑⠭⠑⠍</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>lexem</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>מְלֻכָּה</t>
+        </is>
+      </c>
+      <c r="B19" s="1" t="inlineStr">
+        <is>
+          <t>⠍⠄⠇⠥⠅⠣⠓</t>
+        </is>
+      </c>
+      <c r="C19" s="1" t="inlineStr">
+        <is>
+          <t>m'luk&lt;h</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>מִזְבֵּחַ</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>⠍⠊⠵⠄⠃⠌⠭⠉</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>miz'b/xc</t>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>נְחֹשֶׁת</t>
+        </is>
+      </c>
+      <c r="B20" s="1" t="inlineStr">
+        <is>
+          <t>⠝⠄⠭⠕⠩⠑⠹</t>
+        </is>
+      </c>
+      <c r="C20" s="1" t="inlineStr">
+        <is>
+          <t>n'xo%e?</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>מְלֻכָּה</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>⠍⠄⠇⠥⠅⠣⠓</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>m'luk&lt;h</t>
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>סֵפֶר</t>
+        </is>
+      </c>
+      <c r="B21" s="1" t="inlineStr">
+        <is>
+          <t>⠎⠌⠋⠑⠗</t>
+        </is>
+      </c>
+      <c r="C21" s="1" t="inlineStr">
+        <is>
+          <t>s/fer</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>נְחֹשֶׁת</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>⠝⠄⠭⠕⠩⠑⠹</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>n'xo%e?</t>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>צָפוֹן</t>
+        </is>
+      </c>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>⠮⠣⠋⠪⠝</t>
+        </is>
+      </c>
+      <c r="C22" s="1" t="inlineStr">
+        <is>
+          <t>!&lt;f[n</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>סֵפֶר</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>⠎⠌⠋⠑⠗</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>s/fer</t>
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>קָדוֹשׁ</t>
+        </is>
+      </c>
+      <c r="B23" s="1" t="inlineStr">
+        <is>
+          <t>⠟⠣⠙⠪⠩</t>
+        </is>
+      </c>
+      <c r="C23" s="1" t="inlineStr">
+        <is>
+          <t>q&lt;d[%</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>צָפוֹן</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>⠮⠣⠋⠪⠝</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>!&lt;f[n</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>רוּחַ</t>
+        </is>
+      </c>
+      <c r="B24" s="1" t="inlineStr">
+        <is>
+          <t>⠗⠬⠭⠉</t>
+        </is>
+      </c>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
+          <t>r+xc</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>קָדוֹשׁ</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>⠟⠣⠙⠪⠩</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>q&lt;d[%</t>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>שַׁבָּת</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>⠩⠉⠃⠣⠹</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>%cb&lt;?</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>רוּחַ</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>⠗⠬⠭⠉</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>r+xc</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
-        <is>
-          <t>שַׁבָּת</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>⠩⠉⠃⠣⠹</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>%cb&lt;?</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>שָׂדֶה</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B26" s="1" t="inlineStr">
         <is>
           <t>⠱⠣⠙⠑⠓</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C26" s="1" t="inlineStr">
         <is>
           <t>:&lt;deh</t>
         </is>

</xml_diff>

<commit_message>
fix: wrap the note cells in the Excel workbook
Notes under the tables were single unwrapped cells in the narrow first column, so their text spilled into the empty cells beside them and screen readers reported them as overflowing. The note cells now wrap and align to the top, and the first column of a sheet that carries notes is widened so the wrapped rows stay readable.

Assisted-by: Claude:claude-fable-5
</commit_message>
<xml_diff>
--- a/static/downloads/hebreeuws-braille.xlsx
+++ b/static/downloads/hebreeuws-braille.xlsx
@@ -52,11 +52,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -513,7 +516,7 @@
   <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1331,14 +1334,14 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>De Beet, Kaf, Pee en Tav krijgen in braille een apart teken wanneer zij een Dageesj bevatten. Bij andere consonanten (inclusief de Gimel en Dalet) wordt de Dageesj (braillepunt 5, ⠐) vóór de consonant geplaatst.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1" t="inlineStr">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>De sluitletters in het Hebreeuwse alfabet worden volgens de IHBC-standaard niet onderscheiden van de normale letters.</t>
         </is>
@@ -1361,7 +1364,7 @@
   <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -1694,14 +1697,14 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Leesmoeders</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Wanneer de letters Wav en Jod fungeren als leesmoeders in plaats van als medeklinkers, worden ze tot één enkele braille-cel samengetrokken.</t>
         </is>
@@ -1740,7 +1743,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>ִי</t>
         </is>
@@ -1772,7 +1775,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>ֵי</t>
         </is>
@@ -1804,7 +1807,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>וֹ</t>
         </is>
@@ -1836,7 +1839,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>וּ</t>
         </is>
@@ -1868,7 +1871,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>De letters Alef en Hee worden niet samengetrokken als ze als leesmoeders worden gebruikt.</t>
         </is>
@@ -1892,7 +1895,7 @@
   <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
@@ -2035,14 +2038,14 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Scheidende accenten</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>De onderstaande drie scheidende accenten worden in braille aan het einde van het woord geplaatst waarin ze voorkomen.</t>
         </is>

</xml_diff>